<commit_message>
Fix missing import os in runningvmrscorecard_excel.py; add server deployment notes
</commit_message>
<xml_diff>
--- a/src/template_form.xlsx
+++ b/src/template_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mycatalina-my.sharepoint.com/personal/mjuan_catmktg_com/Documents/Desktop/AIRFLOW_project/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="338" documentId="8_{61384D0D-636B-45CA-95E1-43594CDE4F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{742D9B22-853A-4147-AFEF-4BBD43D90ADF}"/>
+  <xr:revisionPtr revIDLastSave="343" documentId="8_{61384D0D-636B-45CA-95E1-43594CDE4F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7FD82C0-DE89-482F-BB63-C0A11E9E09C8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DA073BC4-92C5-4AC0-B413-FDB045BF64DA}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="146">
   <si>
     <t>ID</t>
   </si>
@@ -454,6 +454,27 @@
   </si>
   <si>
     <t>f6cb4b4e-102e-4a57-a5f6-01d621d10be5</t>
+  </si>
+  <si>
+    <t>PROCTER &amp; GAMBLE COMPANY</t>
+  </si>
+  <si>
+    <t>3.01 WG P&amp;G Mar Scale</t>
+  </si>
+  <si>
+    <t>BL_4810_8050</t>
+  </si>
+  <si>
+    <t>BL_6324_5559</t>
+  </si>
+  <si>
+    <t>1,3</t>
+  </si>
+  <si>
+    <t>69c750c1-f48f-4d60-be80-41073e65cec5</t>
+  </si>
+  <si>
+    <t>4,5,6,7,8,9,10</t>
   </si>
 </sst>
 </file>
@@ -579,8 +600,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D1F2B05-5988-4C2F-96DA-4D766F3F9509}" name="Table1" displayName="Table1" ref="A1:R33" totalsRowShown="0">
-  <autoFilter ref="A1:R33" xr:uid="{4D1F2B05-5988-4C2F-96DA-4D766F3F9509}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D1F2B05-5988-4C2F-96DA-4D766F3F9509}" name="Table1" displayName="Table1" ref="A1:R36" totalsRowShown="0">
+  <autoFilter ref="A1:R36" xr:uid="{4D1F2B05-5988-4C2F-96DA-4D766F3F9509}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{4479560A-E040-45FA-A826-EFE282F586DD}" name="ID" dataDxfId="17">
       <extLst>
@@ -706,7 +727,7 @@
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="nMPdLpYpKkyrl_dnw56hVazLPj-_pJ9FuIH0gDoiyh5URDJWWFRUWkMwTjFEUDFMRDZYSVYxS0NGRC4u" isFormConnected="1" maxResponseId="44" latestEventMarker="100">
+      <xlmsforms:msForm id="nMPdLpYpKkyrl_dnw56hVazLPj-_pJ9FuIH0gDoiyh5URDJWWFRUWkMwTjFEUDFMRDZYSVYxS0NGRC4u" isFormConnected="1" maxResponseId="47" latestEventMarker="101">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -1054,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56C223F4-3877-4B3F-BBCA-AA06221A3262}">
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="18.1796875" customWidth="1"/>
@@ -2599,6 +2620,156 @@
         <v>36</v>
       </c>
       <c r="R33" s="4"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A34" s="4">
+        <v>45</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="M34" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="1">
+        <v>46133</v>
+      </c>
+      <c r="Q34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="R34" s="4"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A35" s="4">
+        <v>46</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+      <c r="P35" s="1">
+        <v>46133</v>
+      </c>
+      <c r="Q35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="R35" s="4"/>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A36" s="4">
+        <v>47</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="M36" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+      <c r="P36" s="1">
+        <v>46133</v>
+      </c>
+      <c r="Q36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="R36" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>